<commit_message>
Schedule: flag 2026-08-19 deploy (v3.8-b7d80dc) on defect sheet + register
Stefan V deployed new Schedule UI to staging (v3.8-da72171/bd246fd ->
v3.8-b7d80dc) after the build-verify findings were recorded. Added a
re-verify banner + per-row 'Re-verify vs 2026-08-19 deploy?' flags to the
tester defect sheet (xlsx Defects to file/Reopen existing tabs + .md), and
a dated SCH-BV-5 row to the outstanding register (Rule 60 layers 1-2;
re-check queued). Docs-only; no TestRail/Jira writes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/schedule/build-verify-2026-08-18/Schedule_Defects-for-Testers_2026-08-19.xlsx
+++ b/build/schedule/build-verify-2026-08-18/Schedule_Defects-for-Testers_2026-08-19.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,8 +49,13 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -60,6 +65,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE699"/>
       </patternFill>
     </fill>
   </fills>
@@ -89,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -102,6 +112,15 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -467,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -481,6 +500,7 @@
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
     <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -497,148 +517,166 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="3" ht="60" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>⚠️ Stefan V deployed NEW Schedule UI changes to staging on 2026-08-19 (build v3.8-b7d80dc), AFTER these findings were recorded (on v3.8-da72171/bd246fd). Some of these may now be FIXED. RE-VERIFY each item on the CURRENT staging build before filing a ticket. A full QA re-check against the new build is queued.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Expected behavior comes from the documented source (spec / epic / PO answer / design), never the build (Standing Rule 57).</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="5"/>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Area</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>Steps to Reproduce</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>Expected behavior</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>Affected TestRail case(s) (C-id + link)</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>Existing ticket (key + status)</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr">
         <is>
           <t>Recommended action</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="K6" s="4" t="inlineStr">
         <is>
           <t>Suggested Jira shape</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="n">
+      <c r="L6" s="9" t="inlineStr">
+        <is>
+          <t>Re-verify vs 2026-08-19 deploy?</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Conflict Detection</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Conflict shifts are styled amber, not red</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>A double-booked (conflicted) shift is highlighted with an amber warning colour and an amber warning icon. The specification says red styling is reserved for conflicts and errors, so a conflict should read as red, not amber.</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>1. Open Schedule.
 2. Find a technician who has two overlapping shifts on the same day (a double-booked / conflict shift — the board already has some, e.g. around Aug 26).
 3. Look at the conflict shift block and its warning icon and note the colour.</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>Conflicts (and errors) are shown in RED. Red styling is reserved for conflicts and errors, and is never used for overtime.</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>Schedule spec v30 §4.11 (styling rule) / §4.12; story SV-8697; epic SV-8685.</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>C30029 (https://shopview.testrail.io/index.php?/cases/view/30029)</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>CREATE NEW Story Defect</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="K7" s="5" t="inlineStr">
         <is>
           <t>Story Defect · parent = the owning story SV-8697 · priority Medium · link owning story SV-8697 'relates to' · no Product Area</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="n">
+      <c r="L7" s="10" t="inlineStr">
+        <is>
+          <t>LIKELY AFFECTED (Stefan: "new Lucide conflict icon everywhere") — re-check the styling/icon before filing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Multi-Day Spread Scheduling</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Multi-day spread dialog cannot read the shop's working hours</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>When you drag a job that needs more than one day, the multi-day spread dialog shows the error "Couldn't read this shop's working hours — reopen to try again." (reproduced on three re-opens). This blocks the spread preview: the "{N} shifts / {total}h" summary, the six how-much options with resolved hours, the start-date default, and the weekend-skip distribution. The schedule board itself resolves the same shop's hours fine (7:00–19:00), so the dialog's own hours lookup is failing where the board's succeeds. It does NOT block ordinary single-day shift creation.
 Note for the tester: this may turn out to be a shop-setup precondition on this shop — please have a dev confirm whether the shop needs explicit business hours configured — but on this build the board reads the hours and the dialog does not.</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>1. Open Schedule on Staging Heavy Duty - 9919.
 2. In the sidebar, find a work order that needs more than one day of work (for example S-9379, about 28.6h remaining).
@@ -646,38 +684,46 @@
 4. Read the multi-day spread dialog.</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>The spread dialog reads the shop's working hours and shows the resolved-hours preview: a "{N} shifts / {total}h" summary, six how-much options with resolved hours, a start date that defaults to the earliest working day, and shifts spread across days skipping weekends only.</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>Schedule spec v30 §4.5 (multi-day spread selector + preview); story SV-8691; epic SV-8685.</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>C29979 (https://shopview.testrail.io/index.php?/cases/view/29979), C29980 (https://shopview.testrail.io/index.php?/cases/view/29980), C29981 (https://shopview.testrail.io/index.php?/cases/view/29981), C29982 (https://shopview.testrail.io/index.php?/cases/view/29982), C29983 (https://shopview.testrail.io/index.php?/cases/view/29983), C29984 (https://shopview.testrail.io/index.php?/cases/view/29984), C43802 (https://shopview.testrail.io/index.php?/cases/view/43802), C43804 (https://shopview.testrail.io/index.php?/cases/view/43804)</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>None found</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>CREATE NEW Story Defect (first have a dev confirm it is not a shop-config precondition)</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
         <is>
           <t>Story Defect · parent = the owning story SV-8691 · priority Medium · link owning story SV-8691 'relates to' · no Product Area</t>
         </is>
       </c>
+      <c r="L8" s="10" t="inlineStr">
+        <is>
+          <t>LIKELY AFFECTED (Stefan: "spread modal single-day plan preview added") — re-check whether it now resolves hours.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:K3"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -688,7 +734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -702,6 +748,7 @@
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
     <col width="34" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -718,90 +765,103 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="3" ht="60" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>⚠️ Stefan V deployed NEW Schedule UI changes to staging on 2026-08-19 (build v3.8-b7d80dc), AFTER these findings were recorded (on v3.8-da72171/bd246fd). Some of these may now be FIXED. RE-VERIFY each item on the CURRENT staging build before filing a ticket. A full QA re-check against the new build is queued.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Expected behavior comes from the documented source (spec / epic / PO answer / design), never the build (Standing Rule 57).</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="5"/>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Area</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>Steps to Reproduce</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>Expected behavior</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>Affected TestRail case(s) (C-id + link)</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>Existing ticket (key + status)</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr">
         <is>
           <t>Recommended action</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="K6" s="4" t="inlineStr">
         <is>
           <t>Suggested Jira shape</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="n">
+      <c r="L6" s="9" t="inlineStr">
+        <is>
+          <t>Re-verify vs 2026-08-19 deploy?</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Drag-and-Drop Scheduling</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>No click-to-arm alternative to dragging a work order</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>There is no way to single-click a sidebar work-order card to "arm" it and then place it on the grid; the only way to schedule is by dragging. The specification's keyboard / accessibility support calls for a click-to-arm alternative. A ticket already captured this (SV-8957) but it is currently closed as Obsolete, and the behaviour still reproduces on the build.</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>1. Open Schedule.
 2. In the sidebar, single-click a work-order card (do not drag it).
@@ -809,96 +869,109 @@
 4. Check whether the work order gets scheduled into that cell.</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>Clicking a work-order card arms it, and clicking a technician cell then places / schedules it — a click-to-arm alternative to dragging (keyboard / accessibility support).</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>Schedule spec v30 §7 (Keyboard support – click-to-arm) / §11 (Accessibility); story SV-8688; epic SV-8685.</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>C29962 (https://shopview.testrail.io/index.php?/cases/view/29962)</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>SV-8957 (OBSOLETE)</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>REOPEN SV-8957 (confirm with Branko that click-to-arm is still required)</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="K7" s="5" t="inlineStr">
         <is>
           <t>Reopen SV-8957. If it must be refiled as new: Story Defect · parent = the owning story SV-8688 · priority Medium · link owning story SV-8688 'relates to' · no Product Area</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="n">
+      <c r="L7" s="10" t="inlineStr">
+        <is>
+          <t>NOT mentioned by Stefan — re-check but likely still reproduces.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Drag-and-Drop Scheduling</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Month view: dragging a work order onto a day does nothing</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>In Month view, dragging a work order from the sidebar onto a day does not create a shift — nothing happens. The same drag in Week view opens the scope picker and works. A ticket captured this (SV-8870) but it is currently closed as Obsolete, and it still reproduces on the build.
 Note for the tester: the specification does not clearly say whether Month view should accept the drop — this is also a question for Branko to confirm the intended Month-view behaviour.</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>1. Open Schedule and switch to Month view.
 2. Drag a work order from the sidebar onto a day cell.
 3. Watch whether a shift is created for that day.</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>Dragging a work order onto a day in Month view creates a shift for that day (the way drag-create works in Week view). Intended Month-view behaviour to be confirmed by Branko.</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>Schedule spec v30 §4.1 (drag-and-drop scheduling) / §4.2 (start-time hierarchy); story SV-8688; epic SV-8685.</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>C43555 (https://shopview.testrail.io/index.php?/cases/view/43555)</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>SV-8870 (OBSOLETE)</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>REOPEN SV-8870 (and confirm with Branko whether Month-view drag-create is intended)</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr">
+      <c r="K8" s="5" t="inlineStr">
         <is>
           <t>Reopen SV-8870. If it must be refiled as new: Story Defect · parent = the owning story SV-8688 · priority Medium · link owning story SV-8688 'relates to' · no Product Area</t>
         </is>
       </c>
+      <c r="L8" s="10" t="inlineStr">
+        <is>
+          <t>LIKELY AFFECTED (Stefan reworked Month view: chips, per-day hover/click) — re-check Month-view drag/interaction.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:K3"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>